<commit_message>
Update meet list excel file
</commit_message>
<xml_diff>
--- a/2025/meet_list_data_ready.xlsx
+++ b/2025/meet_list_data_ready.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dburk\Documents\GitHub\sdxc-data\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943B8C0D-4AC5-4EDC-9695-FEB6BD6B0B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0B361C-7EE0-488D-BC40-03CF376940AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="1560" windowWidth="14400" windowHeight="8904" xr2:uid="{1EB159B1-87E3-4E73-9839-0175057112CF}"/>
+    <workbookView xWindow="4896" yWindow="1692" windowWidth="14400" windowHeight="8904" xr2:uid="{1EB159B1-87E3-4E73-9839-0175057112CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t>official_meet_name</t>
   </si>
@@ -696,13 +696,28 @@
   </si>
   <si>
     <t>dakota12</t>
+  </si>
+  <si>
+    <t>alternative</t>
+  </si>
+  <si>
+    <t>alternative_boys</t>
+  </si>
+  <si>
+    <t>alternative_girls</t>
+  </si>
+  <si>
+    <t>https://sd.milesplit.com/meets/714254-sdhsaa-region-3a-cross-country-meet-2025/results/1232053/raw</t>
+  </si>
+  <si>
+    <t>https://sd.milesplit.com/meets/714254-sdhsaa-region-3a-cross-country-meet-2025/results/1232054/raw</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -720,6 +735,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -748,18 +771,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -767,8 +787,11 @@
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1101,16 +1124,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BABB3D95-ED19-41E8-9BC3-61C8F80036A4}">
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="7"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1146,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>190</v>
       </c>
       <c r="E1" t="s">
@@ -1129,8 +1155,17 @@
       <c r="F1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G1" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1140,7 +1175,7 @@
       <c r="C2" s="2">
         <v>45897</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2">
@@ -1149,8 +1184,11 @@
       <c r="F2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1160,7 +1198,7 @@
       <c r="C3" s="2">
         <v>45897</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>1</v>
       </c>
       <c r="E3">
@@ -1169,8 +1207,11 @@
       <c r="F3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1180,7 +1221,7 @@
       <c r="C4" s="2">
         <v>45897</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4">
@@ -1189,8 +1230,11 @@
       <c r="F4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1200,7 +1244,7 @@
       <c r="C5" s="2">
         <v>45897</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="E5">
@@ -1209,8 +1253,11 @@
       <c r="F5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>191</v>
       </c>
@@ -1220,7 +1267,7 @@
       <c r="C6" s="2">
         <v>45897</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>1</v>
       </c>
       <c r="E6">
@@ -1229,8 +1276,11 @@
       <c r="F6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1240,7 +1290,7 @@
       <c r="C7" s="2">
         <v>45897</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>1</v>
       </c>
       <c r="E7">
@@ -1249,8 +1299,11 @@
       <c r="F7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>193</v>
       </c>
@@ -1260,7 +1313,7 @@
       <c r="C8" s="2">
         <v>45898</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>1</v>
       </c>
       <c r="E8">
@@ -1269,8 +1322,11 @@
       <c r="F8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1280,7 +1336,7 @@
       <c r="C9" s="2">
         <v>45898</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>1</v>
       </c>
       <c r="E9">
@@ -1289,8 +1345,11 @@
       <c r="F9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1300,7 +1359,7 @@
       <c r="C10" s="2">
         <v>45898</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>1</v>
       </c>
       <c r="E10">
@@ -1309,8 +1368,11 @@
       <c r="F10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1320,7 +1382,7 @@
       <c r="C11" s="2">
         <v>45898</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>1</v>
       </c>
       <c r="E11">
@@ -1329,8 +1391,11 @@
       <c r="F11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1340,7 +1405,7 @@
       <c r="C12" s="2">
         <v>45902</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>1</v>
       </c>
       <c r="E12">
@@ -1349,8 +1414,11 @@
       <c r="F12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -1360,7 +1428,7 @@
       <c r="C13" s="2">
         <v>45902</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>1</v>
       </c>
       <c r="E13">
@@ -1369,8 +1437,11 @@
       <c r="F13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1380,7 +1451,7 @@
       <c r="C14" s="2">
         <v>45902</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>1</v>
       </c>
       <c r="E14">
@@ -1389,8 +1460,11 @@
       <c r="F14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1400,7 +1474,7 @@
       <c r="C15" s="2">
         <v>45902</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>1</v>
       </c>
       <c r="E15">
@@ -1409,8 +1483,11 @@
       <c r="F15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>195</v>
       </c>
@@ -1420,7 +1497,7 @@
       <c r="C16" s="2">
         <v>45902</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>1</v>
       </c>
       <c r="E16">
@@ -1429,8 +1506,11 @@
       <c r="F16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1440,7 +1520,7 @@
       <c r="C17" s="2">
         <v>45904</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>1</v>
       </c>
       <c r="E17">
@@ -1449,8 +1529,11 @@
       <c r="F17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -1460,7 +1543,7 @@
       <c r="C18" s="2">
         <v>45905</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>1</v>
       </c>
       <c r="E18">
@@ -1469,8 +1552,11 @@
       <c r="F18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>197</v>
       </c>
@@ -1480,7 +1566,7 @@
       <c r="C19" s="2">
         <v>45905</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>1</v>
       </c>
       <c r="E19">
@@ -1489,8 +1575,11 @@
       <c r="F19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -1500,7 +1589,7 @@
       <c r="C20" s="2">
         <v>45905</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>1</v>
       </c>
       <c r="E20">
@@ -1509,8 +1598,11 @@
       <c r="F20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -1520,7 +1612,7 @@
       <c r="C21" s="2">
         <v>45905</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>1</v>
       </c>
       <c r="E21">
@@ -1529,8 +1621,11 @@
       <c r="F21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -1540,7 +1635,7 @@
       <c r="C22" s="2">
         <v>45906</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>1</v>
       </c>
       <c r="E22">
@@ -1549,8 +1644,11 @@
       <c r="F22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G22" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1560,7 +1658,7 @@
       <c r="C23" s="2">
         <v>45908</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>2</v>
       </c>
       <c r="E23">
@@ -1569,8 +1667,11 @@
       <c r="F23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -1580,7 +1681,7 @@
       <c r="C24" s="2">
         <v>45909</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>2</v>
       </c>
       <c r="E24">
@@ -1589,8 +1690,11 @@
       <c r="F24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>201</v>
       </c>
@@ -1600,7 +1704,7 @@
       <c r="C25" s="2">
         <v>45909</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>2</v>
       </c>
       <c r="E25">
@@ -1609,8 +1713,11 @@
       <c r="F25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -1620,7 +1727,7 @@
       <c r="C26" s="2">
         <v>45909</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <v>2</v>
       </c>
       <c r="E26">
@@ -1629,28 +1736,34 @@
       <c r="F26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="6" t="s">
+      <c r="G26" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="5">
         <v>45910</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="6">
         <v>2</v>
       </c>
-      <c r="E27" s="6">
-        <v>1</v>
-      </c>
-      <c r="F27" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E27" s="4">
+        <v>1</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
+      <c r="G27" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>199</v>
       </c>
@@ -1660,7 +1773,7 @@
       <c r="C28" s="2">
         <v>45910</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="3">
         <v>2</v>
       </c>
       <c r="E28">
@@ -1669,8 +1782,11 @@
       <c r="F28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -1680,7 +1796,7 @@
       <c r="C29" s="2">
         <v>45911</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="3">
         <v>2</v>
       </c>
       <c r="E29">
@@ -1689,8 +1805,11 @@
       <c r="F29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>50</v>
       </c>
@@ -1700,7 +1819,7 @@
       <c r="C30" s="2">
         <v>45911</v>
       </c>
-      <c r="D30" s="4">
+      <c r="D30" s="3">
         <v>2</v>
       </c>
       <c r="E30">
@@ -1709,8 +1828,11 @@
       <c r="F30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1720,7 +1842,7 @@
       <c r="C31" s="2">
         <v>45911</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D31" s="3">
         <v>2</v>
       </c>
       <c r="E31">
@@ -1729,8 +1851,11 @@
       <c r="F31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>54</v>
       </c>
@@ -1740,7 +1865,7 @@
       <c r="C32" s="2">
         <v>45912</v>
       </c>
-      <c r="D32" s="4">
+      <c r="D32" s="3">
         <v>2</v>
       </c>
       <c r="E32">
@@ -1749,8 +1874,11 @@
       <c r="F32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>56</v>
       </c>
@@ -1760,7 +1888,7 @@
       <c r="C33" s="2">
         <v>45913</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="3">
         <v>2</v>
       </c>
       <c r="E33">
@@ -1769,8 +1897,11 @@
       <c r="F33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>58</v>
       </c>
@@ -1780,7 +1911,7 @@
       <c r="C34" s="2">
         <v>45913</v>
       </c>
-      <c r="D34" s="4">
+      <c r="D34" s="3">
         <v>2</v>
       </c>
       <c r="E34">
@@ -1789,8 +1920,11 @@
       <c r="F34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>60</v>
       </c>
@@ -1800,7 +1934,7 @@
       <c r="C35" s="2">
         <v>45913</v>
       </c>
-      <c r="D35" s="4">
+      <c r="D35" s="3">
         <v>2</v>
       </c>
       <c r="E35">
@@ -1809,8 +1943,11 @@
       <c r="F35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>198</v>
       </c>
@@ -1820,7 +1957,7 @@
       <c r="C36" s="2">
         <v>45913</v>
       </c>
-      <c r="D36" s="4">
+      <c r="D36" s="3">
         <v>2</v>
       </c>
       <c r="E36">
@@ -1829,8 +1966,11 @@
       <c r="F36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G36" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>62</v>
       </c>
@@ -1840,7 +1980,7 @@
       <c r="C37" s="2">
         <v>45915</v>
       </c>
-      <c r="D37" s="4">
+      <c r="D37" s="3">
         <v>3</v>
       </c>
       <c r="E37">
@@ -1849,8 +1989,11 @@
       <c r="F37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>64</v>
       </c>
@@ -1869,8 +2012,11 @@
       <c r="F38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>66</v>
       </c>
@@ -1880,7 +2026,7 @@
       <c r="C39" s="2">
         <v>45915</v>
       </c>
-      <c r="D39" s="4">
+      <c r="D39" s="3">
         <v>3</v>
       </c>
       <c r="E39">
@@ -1889,8 +2035,11 @@
       <c r="F39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>68</v>
       </c>
@@ -1900,7 +2049,7 @@
       <c r="C40" s="2">
         <v>45915</v>
       </c>
-      <c r="D40" s="4">
+      <c r="D40" s="3">
         <v>3</v>
       </c>
       <c r="E40">
@@ -1909,8 +2058,11 @@
       <c r="F40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>185</v>
       </c>
@@ -1920,7 +2072,7 @@
       <c r="C41" s="2">
         <v>45915</v>
       </c>
-      <c r="D41" s="4">
+      <c r="D41" s="3">
         <v>3</v>
       </c>
       <c r="E41">
@@ -1929,8 +2081,11 @@
       <c r="F41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>70</v>
       </c>
@@ -1940,7 +2095,7 @@
       <c r="C42" s="2">
         <v>45917</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D42" s="3">
         <v>3</v>
       </c>
       <c r="E42">
@@ -1949,8 +2104,11 @@
       <c r="F42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>88</v>
       </c>
@@ -1960,7 +2118,7 @@
       <c r="C43" s="2">
         <v>45917</v>
       </c>
-      <c r="D43" s="4">
+      <c r="D43" s="3">
         <v>3</v>
       </c>
       <c r="E43">
@@ -1969,8 +2127,11 @@
       <c r="F43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G43" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>72</v>
       </c>
@@ -1980,7 +2141,7 @@
       <c r="C44" s="2">
         <v>45918</v>
       </c>
-      <c r="D44" s="4">
+      <c r="D44" s="3">
         <v>3</v>
       </c>
       <c r="E44">
@@ -1989,8 +2150,11 @@
       <c r="F44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>74</v>
       </c>
@@ -2000,7 +2164,7 @@
       <c r="C45" s="2">
         <v>45920</v>
       </c>
-      <c r="D45" s="4">
+      <c r="D45" s="3">
         <v>3</v>
       </c>
       <c r="E45">
@@ -2009,8 +2173,11 @@
       <c r="F45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G45" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>76</v>
       </c>
@@ -2020,7 +2187,7 @@
       <c r="C46" s="2">
         <v>45920</v>
       </c>
-      <c r="D46" s="4">
+      <c r="D46" s="3">
         <v>3</v>
       </c>
       <c r="E46">
@@ -2029,8 +2196,11 @@
       <c r="F46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>78</v>
       </c>
@@ -2040,7 +2210,7 @@
       <c r="C47" s="2">
         <v>45922</v>
       </c>
-      <c r="D47" s="4">
+      <c r="D47" s="3">
         <v>4</v>
       </c>
       <c r="E47">
@@ -2049,8 +2219,11 @@
       <c r="F47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G47" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>80</v>
       </c>
@@ -2060,7 +2233,7 @@
       <c r="C48" s="2">
         <v>45922</v>
       </c>
-      <c r="D48" s="4">
+      <c r="D48" s="3">
         <v>4</v>
       </c>
       <c r="E48">
@@ -2069,8 +2242,11 @@
       <c r="F48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G48" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>82</v>
       </c>
@@ -2080,7 +2256,7 @@
       <c r="C49" s="2">
         <v>45922</v>
       </c>
-      <c r="D49" s="4">
+      <c r="D49" s="3">
         <v>4</v>
       </c>
       <c r="E49">
@@ -2089,8 +2265,11 @@
       <c r="F49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G49" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>84</v>
       </c>
@@ -2100,7 +2279,7 @@
       <c r="C50" s="2">
         <v>45922</v>
       </c>
-      <c r="D50" s="4">
+      <c r="D50" s="3">
         <v>4</v>
       </c>
       <c r="E50">
@@ -2109,8 +2288,11 @@
       <c r="F50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>203</v>
       </c>
@@ -2120,7 +2302,7 @@
       <c r="C51" s="2">
         <v>45922</v>
       </c>
-      <c r="D51" s="4">
+      <c r="D51" s="3">
         <v>4</v>
       </c>
       <c r="E51">
@@ -2129,8 +2311,11 @@
       <c r="F51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>45</v>
       </c>
@@ -2140,7 +2325,7 @@
       <c r="C52" s="2">
         <v>45924</v>
       </c>
-      <c r="D52" s="4">
+      <c r="D52" s="3">
         <v>4</v>
       </c>
       <c r="E52">
@@ -2149,8 +2334,11 @@
       <c r="F52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G52" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>86</v>
       </c>
@@ -2160,7 +2348,7 @@
       <c r="C53" s="2">
         <v>45924</v>
       </c>
-      <c r="D53" s="4">
+      <c r="D53" s="3">
         <v>4</v>
       </c>
       <c r="E53">
@@ -2169,8 +2357,11 @@
       <c r="F53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G53" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>112</v>
       </c>
@@ -2180,7 +2371,7 @@
       <c r="C54" s="2">
         <v>45924</v>
       </c>
-      <c r="D54" s="4">
+      <c r="D54" s="3">
         <v>4</v>
       </c>
       <c r="E54">
@@ -2189,8 +2380,11 @@
       <c r="F54">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G54" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>87</v>
       </c>
@@ -2200,7 +2394,7 @@
       <c r="C55" s="2">
         <v>45924</v>
       </c>
-      <c r="D55" s="4">
+      <c r="D55" s="3">
         <v>4</v>
       </c>
       <c r="E55">
@@ -2209,8 +2403,11 @@
       <c r="F55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G55" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>91</v>
       </c>
@@ -2220,7 +2417,7 @@
       <c r="C56" s="2">
         <v>45925</v>
       </c>
-      <c r="D56" s="4">
+      <c r="D56" s="3">
         <v>4</v>
       </c>
       <c r="E56">
@@ -2229,8 +2426,11 @@
       <c r="F56">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G56" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>92</v>
       </c>
@@ -2240,7 +2440,7 @@
       <c r="C57" s="2">
         <v>45925</v>
       </c>
-      <c r="D57" s="4">
+      <c r="D57" s="3">
         <v>4</v>
       </c>
       <c r="E57">
@@ -2249,8 +2449,11 @@
       <c r="F57">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G57" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>93</v>
       </c>
@@ -2260,7 +2463,7 @@
       <c r="C58" s="2">
         <v>45925</v>
       </c>
-      <c r="D58" s="4">
+      <c r="D58" s="3">
         <v>4</v>
       </c>
       <c r="E58">
@@ -2269,8 +2472,11 @@
       <c r="F58">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G58" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>94</v>
       </c>
@@ -2280,7 +2486,7 @@
       <c r="C59" s="2">
         <v>45925</v>
       </c>
-      <c r="D59" s="4">
+      <c r="D59" s="3">
         <v>4</v>
       </c>
       <c r="E59">
@@ -2289,8 +2495,11 @@
       <c r="F59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G59" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>99</v>
       </c>
@@ -2300,7 +2509,7 @@
       <c r="C60" s="2">
         <v>45926</v>
       </c>
-      <c r="D60" s="4">
+      <c r="D60" s="3">
         <v>4</v>
       </c>
       <c r="E60">
@@ -2309,8 +2518,11 @@
       <c r="F60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G60" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>206</v>
       </c>
@@ -2320,7 +2532,7 @@
       <c r="C61" s="2">
         <v>45927</v>
       </c>
-      <c r="D61" s="4">
+      <c r="D61" s="3">
         <v>4</v>
       </c>
       <c r="E61">
@@ -2329,8 +2541,11 @@
       <c r="F61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G61" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>101</v>
       </c>
@@ -2340,7 +2555,7 @@
       <c r="C62" s="2">
         <v>45927</v>
       </c>
-      <c r="D62" s="4">
+      <c r="D62" s="3">
         <v>4</v>
       </c>
       <c r="E62">
@@ -2349,8 +2564,11 @@
       <c r="F62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G62" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>107</v>
       </c>
@@ -2360,7 +2578,7 @@
       <c r="C63" s="2">
         <v>45929</v>
       </c>
-      <c r="D63" s="4">
+      <c r="D63" s="3">
         <v>5</v>
       </c>
       <c r="E63">
@@ -2369,8 +2587,11 @@
       <c r="F63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G63" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>209</v>
       </c>
@@ -2380,7 +2601,7 @@
       <c r="C64" s="2">
         <v>45929</v>
       </c>
-      <c r="D64" s="4">
+      <c r="D64" s="3">
         <v>5</v>
       </c>
       <c r="E64">
@@ -2389,8 +2610,11 @@
       <c r="F64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G64" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>106</v>
       </c>
@@ -2400,7 +2624,7 @@
       <c r="C65" s="2">
         <v>45929</v>
       </c>
-      <c r="D65" s="4">
+      <c r="D65" s="3">
         <v>5</v>
       </c>
       <c r="E65">
@@ -2409,8 +2633,11 @@
       <c r="F65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G65" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>108</v>
       </c>
@@ -2420,7 +2647,7 @@
       <c r="C66" s="2">
         <v>45929</v>
       </c>
-      <c r="D66" s="4">
+      <c r="D66" s="3">
         <v>5</v>
       </c>
       <c r="E66">
@@ -2429,8 +2656,11 @@
       <c r="F66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G66" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>109</v>
       </c>
@@ -2440,7 +2670,7 @@
       <c r="C67" s="2">
         <v>45930</v>
       </c>
-      <c r="D67" s="4">
+      <c r="D67" s="3">
         <v>5</v>
       </c>
       <c r="E67">
@@ -2449,8 +2679,11 @@
       <c r="F67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G67" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>110</v>
       </c>
@@ -2460,7 +2693,7 @@
       <c r="C68" s="2">
         <v>45930</v>
       </c>
-      <c r="D68" s="4">
+      <c r="D68" s="3">
         <v>5</v>
       </c>
       <c r="E68">
@@ -2469,8 +2702,11 @@
       <c r="F68">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G68" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>111</v>
       </c>
@@ -2480,7 +2716,7 @@
       <c r="C69" s="2">
         <v>45931</v>
       </c>
-      <c r="D69" s="4">
+      <c r="D69" s="3">
         <v>5</v>
       </c>
       <c r="E69">
@@ -2489,8 +2725,11 @@
       <c r="F69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G69" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>116</v>
       </c>
@@ -2500,7 +2739,7 @@
       <c r="C70" s="2">
         <v>45932</v>
       </c>
-      <c r="D70" s="4">
+      <c r="D70" s="3">
         <v>5</v>
       </c>
       <c r="E70">
@@ -2509,8 +2748,11 @@
       <c r="F70">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G70" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>118</v>
       </c>
@@ -2520,7 +2762,7 @@
       <c r="C71" s="2">
         <v>45932</v>
       </c>
-      <c r="D71" s="4">
+      <c r="D71" s="3">
         <v>5</v>
       </c>
       <c r="E71">
@@ -2529,8 +2771,11 @@
       <c r="F71">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G71" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>119</v>
       </c>
@@ -2540,7 +2785,7 @@
       <c r="C72" s="2">
         <v>45932</v>
       </c>
-      <c r="D72" s="4">
+      <c r="D72" s="3">
         <v>5</v>
       </c>
       <c r="E72">
@@ -2549,8 +2794,11 @@
       <c r="F72">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G72" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>120</v>
       </c>
@@ -2560,7 +2808,7 @@
       <c r="C73" s="2">
         <v>45932</v>
       </c>
-      <c r="D73" s="4">
+      <c r="D73" s="3">
         <v>5</v>
       </c>
       <c r="E73">
@@ -2569,8 +2817,11 @@
       <c r="F73">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G73" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>153</v>
       </c>
@@ -2580,7 +2831,7 @@
       <c r="C74" s="2">
         <v>45933</v>
       </c>
-      <c r="D74" s="4">
+      <c r="D74" s="3">
         <v>5</v>
       </c>
       <c r="E74">
@@ -2589,8 +2840,11 @@
       <c r="F74">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G74" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>124</v>
       </c>
@@ -2600,7 +2854,7 @@
       <c r="C75" s="2">
         <v>45934</v>
       </c>
-      <c r="D75" s="4">
+      <c r="D75" s="3">
         <v>5</v>
       </c>
       <c r="E75">
@@ -2609,8 +2863,11 @@
       <c r="F75">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G75" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>125</v>
       </c>
@@ -2620,7 +2877,7 @@
       <c r="C76" s="2">
         <v>45934</v>
       </c>
-      <c r="D76" s="4">
+      <c r="D76" s="3">
         <v>5</v>
       </c>
       <c r="E76">
@@ -2629,8 +2886,11 @@
       <c r="F76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G76" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>130</v>
       </c>
@@ -2640,7 +2900,7 @@
       <c r="C77" s="2">
         <v>45936</v>
       </c>
-      <c r="D77" s="4">
+      <c r="D77" s="3">
         <v>6</v>
       </c>
       <c r="E77">
@@ -2649,8 +2909,11 @@
       <c r="F77">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G77" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>129</v>
       </c>
@@ -2660,7 +2923,7 @@
       <c r="C78" s="2">
         <v>45936</v>
       </c>
-      <c r="D78" s="4">
+      <c r="D78" s="3">
         <v>6</v>
       </c>
       <c r="E78">
@@ -2669,8 +2932,11 @@
       <c r="F78">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G78" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>131</v>
       </c>
@@ -2680,7 +2946,7 @@
       <c r="C79" s="2">
         <v>45936</v>
       </c>
-      <c r="D79" s="4">
+      <c r="D79" s="3">
         <v>6</v>
       </c>
       <c r="E79">
@@ -2689,8 +2955,11 @@
       <c r="F79">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G79" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>132</v>
       </c>
@@ -2700,7 +2969,7 @@
       <c r="C80" s="2">
         <v>45936</v>
       </c>
-      <c r="D80" s="4">
+      <c r="D80" s="3">
         <v>6</v>
       </c>
       <c r="E80">
@@ -2709,8 +2978,11 @@
       <c r="F80">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G80" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>137</v>
       </c>
@@ -2720,7 +2992,7 @@
       <c r="C81" s="2">
         <v>45937</v>
       </c>
-      <c r="D81" s="4">
+      <c r="D81" s="3">
         <v>6</v>
       </c>
       <c r="E81">
@@ -2729,8 +3001,11 @@
       <c r="F81">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G81" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>138</v>
       </c>
@@ -2740,7 +3015,7 @@
       <c r="C82" s="2">
         <v>45938</v>
       </c>
-      <c r="D82" s="4">
+      <c r="D82" s="3">
         <v>6</v>
       </c>
       <c r="E82">
@@ -2749,8 +3024,11 @@
       <c r="F82">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G82" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>216</v>
       </c>
@@ -2760,7 +3038,7 @@
       <c r="C83" s="2">
         <v>45938</v>
       </c>
-      <c r="D83" s="4">
+      <c r="D83" s="3">
         <v>6</v>
       </c>
       <c r="E83">
@@ -2769,8 +3047,11 @@
       <c r="F83">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G83" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>210</v>
       </c>
@@ -2780,7 +3061,7 @@
       <c r="C84" s="2">
         <v>45938</v>
       </c>
-      <c r="D84" s="4">
+      <c r="D84" s="3">
         <v>6</v>
       </c>
       <c r="E84">
@@ -2789,8 +3070,11 @@
       <c r="F84">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G84" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>140</v>
       </c>
@@ -2800,7 +3084,7 @@
       <c r="C85" s="2">
         <v>45938</v>
       </c>
-      <c r="D85" s="4">
+      <c r="D85" s="3">
         <v>6</v>
       </c>
       <c r="E85">
@@ -2809,8 +3093,11 @@
       <c r="F85">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G85" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>141</v>
       </c>
@@ -2820,7 +3107,7 @@
       <c r="C86" s="2">
         <v>45939</v>
       </c>
-      <c r="D86" s="4">
+      <c r="D86" s="3">
         <v>6</v>
       </c>
       <c r="E86">
@@ -2829,8 +3116,11 @@
       <c r="F86">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G86" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>142</v>
       </c>
@@ -2840,7 +3130,7 @@
       <c r="C87" s="2">
         <v>45939</v>
       </c>
-      <c r="D87" s="4">
+      <c r="D87" s="3">
         <v>6</v>
       </c>
       <c r="E87">
@@ -2849,8 +3139,11 @@
       <c r="F87">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G87" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>143</v>
       </c>
@@ -2860,7 +3153,7 @@
       <c r="C88" s="2">
         <v>45939</v>
       </c>
-      <c r="D88" s="4">
+      <c r="D88" s="3">
         <v>6</v>
       </c>
       <c r="E88">
@@ -2869,8 +3162,11 @@
       <c r="F88">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G88" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>144</v>
       </c>
@@ -2880,7 +3176,7 @@
       <c r="C89" s="2">
         <v>45939</v>
       </c>
-      <c r="D89" s="4">
+      <c r="D89" s="3">
         <v>6</v>
       </c>
       <c r="E89">
@@ -2889,8 +3185,11 @@
       <c r="F89">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G89" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>145</v>
       </c>
@@ -2900,7 +3199,7 @@
       <c r="C90" s="2">
         <v>45939</v>
       </c>
-      <c r="D90" s="4">
+      <c r="D90" s="3">
         <v>6</v>
       </c>
       <c r="E90">
@@ -2909,8 +3208,11 @@
       <c r="F90">
         <v>0</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G90" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>146</v>
       </c>
@@ -2920,7 +3222,7 @@
       <c r="C91" s="2">
         <v>45939</v>
       </c>
-      <c r="D91" s="4">
+      <c r="D91" s="3">
         <v>6</v>
       </c>
       <c r="E91">
@@ -2929,8 +3231,11 @@
       <c r="F91">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G91" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>152</v>
       </c>
@@ -2940,7 +3245,7 @@
       <c r="C92" s="2">
         <v>45941</v>
       </c>
-      <c r="D92" s="4">
+      <c r="D92" s="3">
         <v>6</v>
       </c>
       <c r="E92">
@@ -2949,8 +3254,11 @@
       <c r="F92">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G92" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>157</v>
       </c>
@@ -2960,7 +3268,7 @@
       <c r="C93" s="2">
         <v>45945</v>
       </c>
-      <c r="D93" s="4">
+      <c r="D93" s="3">
         <v>7</v>
       </c>
       <c r="E93">
@@ -2969,8 +3277,11 @@
       <c r="F93">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G93" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>162</v>
       </c>
@@ -2980,7 +3291,7 @@
       <c r="C94" s="2">
         <v>45945</v>
       </c>
-      <c r="D94" s="4">
+      <c r="D94" s="3">
         <v>7</v>
       </c>
       <c r="E94">
@@ -2989,8 +3300,11 @@
       <c r="F94">
         <v>0</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G94" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>158</v>
       </c>
@@ -3000,7 +3314,7 @@
       <c r="C95" s="2">
         <v>45945</v>
       </c>
-      <c r="D95" s="4">
+      <c r="D95" s="3">
         <v>7</v>
       </c>
       <c r="E95">
@@ -3009,8 +3323,11 @@
       <c r="F95">
         <v>0</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G95" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>163</v>
       </c>
@@ -3020,7 +3337,7 @@
       <c r="C96" s="2">
         <v>45945</v>
       </c>
-      <c r="D96" s="4">
+      <c r="D96" s="3">
         <v>7</v>
       </c>
       <c r="E96">
@@ -3029,8 +3346,11 @@
       <c r="F96">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G96" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>164</v>
       </c>
@@ -3040,7 +3360,7 @@
       <c r="C97" s="2">
         <v>45945</v>
       </c>
-      <c r="D97" s="4">
+      <c r="D97" s="3">
         <v>7</v>
       </c>
       <c r="E97">
@@ -3049,8 +3369,11 @@
       <c r="F97">
         <v>0</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G97" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>165</v>
       </c>
@@ -3060,7 +3383,7 @@
       <c r="C98" s="2">
         <v>45945</v>
       </c>
-      <c r="D98" s="4">
+      <c r="D98" s="3">
         <v>7</v>
       </c>
       <c r="E98">
@@ -3069,8 +3392,11 @@
       <c r="F98">
         <v>0</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G98" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>166</v>
       </c>
@@ -3080,7 +3406,7 @@
       <c r="C99" s="2">
         <v>45945</v>
       </c>
-      <c r="D99" s="4">
+      <c r="D99" s="3">
         <v>7</v>
       </c>
       <c r="E99">
@@ -3089,28 +3415,34 @@
       <c r="F99">
         <v>0</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="1" t="s">
+      <c r="G99" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
         <v>177</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" t="s">
         <v>178</v>
       </c>
-      <c r="C100" s="3">
+      <c r="C100" s="2">
         <v>45946</v>
       </c>
-      <c r="D100" s="5">
+      <c r="D100" s="3">
         <v>7</v>
       </c>
-      <c r="E100" s="1">
+      <c r="E100">
         <v>1</v>
       </c>
       <c r="F100">
         <v>0</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G100" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>212</v>
       </c>
@@ -3120,17 +3452,20 @@
       <c r="C101" s="2">
         <v>45946</v>
       </c>
-      <c r="D101" s="4">
+      <c r="D101" s="3">
         <v>7</v>
       </c>
       <c r="E101">
         <v>1</v>
       </c>
       <c r="F101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="G101" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>155</v>
       </c>
@@ -3140,7 +3475,7 @@
       <c r="C102" s="2">
         <v>45946</v>
       </c>
-      <c r="D102" s="4">
+      <c r="D102" s="3">
         <v>7</v>
       </c>
       <c r="E102">
@@ -3149,8 +3484,11 @@
       <c r="F102">
         <v>0</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G102" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>159</v>
       </c>
@@ -3160,7 +3498,7 @@
       <c r="C103" s="2">
         <v>45946</v>
       </c>
-      <c r="D103" s="4">
+      <c r="D103" s="3">
         <v>7</v>
       </c>
       <c r="E103">
@@ -3169,8 +3507,17 @@
       <c r="F103">
         <v>0</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G103" s="7">
+        <v>1</v>
+      </c>
+      <c r="H103" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="I103" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>160</v>
       </c>
@@ -3180,7 +3527,7 @@
       <c r="C104" s="2">
         <v>45946</v>
       </c>
-      <c r="D104" s="4">
+      <c r="D104" s="3">
         <v>7</v>
       </c>
       <c r="E104">
@@ -3189,8 +3536,11 @@
       <c r="F104">
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G104" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>161</v>
       </c>
@@ -3200,7 +3550,7 @@
       <c r="C105" s="2">
         <v>45946</v>
       </c>
-      <c r="D105" s="4">
+      <c r="D105" s="3">
         <v>7</v>
       </c>
       <c r="E105">
@@ -3209,8 +3559,11 @@
       <c r="F105">
         <v>0</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G105" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>180</v>
       </c>
@@ -3220,7 +3573,7 @@
       <c r="C106" s="2">
         <v>45955</v>
       </c>
-      <c r="D106" s="4">
+      <c r="D106" s="3">
         <v>8</v>
       </c>
       <c r="E106">
@@ -3229,8 +3582,11 @@
       <c r="F106">
         <v>0</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G106" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>179</v>
       </c>
@@ -3240,7 +3596,7 @@
       <c r="C107" s="2">
         <v>45955</v>
       </c>
-      <c r="D107" s="4">
+      <c r="D107" s="3">
         <v>8</v>
       </c>
       <c r="E107">
@@ -3249,8 +3605,11 @@
       <c r="F107">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G107" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>181</v>
       </c>
@@ -3260,13 +3619,16 @@
       <c r="C108" s="2">
         <v>228576</v>
       </c>
-      <c r="D108" s="4">
+      <c r="D108" s="3">
         <v>8</v>
       </c>
       <c r="E108">
         <v>1</v>
       </c>
       <c r="F108">
+        <v>0</v>
+      </c>
+      <c r="G108" s="7">
         <v>0</v>
       </c>
     </row>
@@ -3275,6 +3637,9 @@
     <sortCondition ref="C2:C117"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="H103" r:id="rId1" xr:uid="{D6A8393A-79A8-4A90-8D9D-62BAA5936E48}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>